<commit_message>
added KB0050 re camera power
</commit_message>
<xml_diff>
--- a/knowledgebase.xlsx
+++ b/knowledgebase.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{341CE5BD-3C0E-F449-81F9-D9345DDCFC93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86C401D9-7412-4A4A-951A-BE8123222D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46440" yWindow="-29880" windowWidth="55380" windowHeight="36160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Issues" sheetId="1" r:id="rId1"/>
     <sheet name="Metadata" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="549">
   <si>
     <t xml:space="preserve"> IssueID </t>
   </si>
@@ -1798,6 +1798,36 @@
 4) Reboot CUMU-E001 and re-establish the Reaper session.
 5) Using the Q-SYS touchpad (2408-2704) or the app on CUMU-E001, set 'Video Send' back to 'DAW'."
 If situation continues to occur, consider switching the video source to Matrix. You can actively mix the inputs using the matrix mix on dlive director.  </t>
+  </si>
+  <si>
+    <t>KB0050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video camera does not respond to power on. </t>
+  </si>
+  <si>
+    <t>When operator presses the power on sequence, the camera does not respond.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When starting up for an event and going through the power on seqeunce a camera does not respoond the the power on request. </t>
+  </si>
+  <si>
+    <t>Unknown.</t>
+  </si>
+  <si>
+    <t>We need to power cycle the camera. Cameras 1 and 2 are powered via the network cable (PoE) and Camera 3 should be the same but is currently different. 
+For cameras 1 or 2, we need to located the correct camera network cable and unplug it, wait 10 seconds and then plug it back in. This can be done from the camera end or the network swtich end. For the camera end you need to stand up on the pews to be able to reach the network cable. Not always easy. 
+Doing the same operation at the network switch end is physically easier but you have to find the right cable. At the moment (september 2026) the cameras are all pluggged into network swtich NSCU-A004, Camera 1 is in port 1, 2 in 2 and 3 in 3. (In the future the connection will be moved to swtich 2603-1203 (in the large cabinet in the corner, ports yet to be determined)
+Camera 3 is not currently powered via the network, but rather by the power cable over the edge of the baclony. The audio system must be on for camera 3 to work. To power cycle .camera 3, unplug its power cord.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZVCU- A001,ZVCU- A002, ZVCU- A003 </t>
+  </si>
+  <si>
+    <t>#camera, #video, #power</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seems to occur mostly with camera 1. </t>
   </si>
 </sst>
 </file>
@@ -1978,13 +2008,13 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2057,8 +2087,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}" name="Table1" displayName="Table1" ref="A1:O50" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
-  <autoFilter ref="A1:O50" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}" name="Table1" displayName="Table1" ref="A1:O51" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+  <autoFilter ref="A1:O51" xr:uid="{8DA13CB4-8680-0D4C-A016-6564C2E20834}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O40">
     <sortCondition ref="A2:A40"/>
   </sortState>
@@ -2400,7 +2430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="1" customWidth="1"/>
@@ -4551,7 +4581,7 @@
       </c>
       <c r="O49" s="4"/>
     </row>
-    <row r="50" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:15" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>535</v>
       </c>
@@ -4596,6 +4626,53 @@
       </c>
       <c r="O50" s="4" t="s">
         <v>537</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A51" s="4" t="s">
+        <v>540</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>541</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>545</v>
+      </c>
+      <c r="I51" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="J51" s="4" t="s">
+        <v>546</v>
+      </c>
+      <c r="K51" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="L51" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="M51" s="4">
+        <v>51</v>
+      </c>
+      <c r="N51" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O51" s="4" t="s">
+        <v>548</v>
       </c>
     </row>
   </sheetData>
@@ -5156,7 +5233,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A9" s="10" t="s">
         <v>7</v>
       </c>
@@ -5180,7 +5257,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
         <v>10</v>
       </c>
@@ -5212,7 +5289,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="68" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>14</v>
       </c>

</xml_diff>